<commit_message>
Update ELSTAT data for 2025
</commit_message>
<xml_diff>
--- a/data_prep/ELSTAT/SBR03_01.xlsx
+++ b/data_prep/ELSTAT/SBR03_01.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dstamou\Documents\REGISTERS AND BIG ENTERPRISES\NEW COVID 19 DT\55 56_2025\ΙΟΥΝΙΟΣ\ΠΙΝΑΚΕΣ ΙΣΤΟΣΕΛΙΔΑΣ\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\03_ΤΜΗΜΑ ΜΗΤΡΩΩΝ ΚΑΙ ΜΕΓΑΛΩΝ ΕΠΙΧΕΙΡΗΣΕΩΝ\BUSINESS REGISTER\1_PR_COVID_NACE_55_56_2025\Q4_2025\ΠΙΝΑΚΕΣ ΙΣΤΟΣΕΛΙΔΑΣ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5F3B456-B879-4EE0-84D0-458857CC1387}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A50C00F3-D342-4EB4-9D25-CA54198F2780}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-113" yWindow="-113" windowWidth="24267" windowHeight="13311" activeTab="1" xr2:uid="{DA990AAA-CAE0-4CF1-9D21-45B7EAEB1E8F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{DA990AAA-CAE0-4CF1-9D21-45B7EAEB1E8F}"/>
   </bookViews>
   <sheets>
     <sheet name="NACE_55_A" sheetId="2" r:id="rId1"/>
@@ -41,16 +41,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="119">
   <si>
     <t>ΠΕΡΙΦΕΡΕΙΑ</t>
   </si>
   <si>
     <t>ΠΕΡΙΦΕΡΕΙΑΚΗ ΕΝΟΤΗΤΑ</t>
-  </si>
-  <si>
-    <t>ΚΥΚΛΟΣ ΕΡΓΑΣΙΩΝ
-(σε ευρώ)</t>
   </si>
   <si>
     <t>ΑΝΑΤΟΛΙΚΗΣ ΜΑΚΕΔΟΝΙΑΣ ΚΑΙ ΘΡΑΚΗΣ</t>
@@ -693,7 +689,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -820,11 +816,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="hair">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -872,6 +881,9 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -890,11 +902,14 @@
     <xf numFmtId="0" fontId="13" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -902,10 +917,8 @@
     <xf numFmtId="0" fontId="13" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -926,7 +939,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Κανονικό" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -942,7 +955,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Θέμα Office 2013 - 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
@@ -1239,25 +1252,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EC57FCF-9924-42BC-B6FB-E6A79A0D85EC}">
   <dimension ref="A1:N78"/>
-  <sheetFormatPr defaultRowHeight="15.05" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.5546875" customWidth="1"/>
     <col min="2" max="2" width="15.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="7" width="16.33203125" customWidth="1"/>
     <col min="8" max="8" width="16.44140625" customWidth="1"/>
+    <col min="9" max="9" width="16.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="52.3" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="17" t="s">
-        <v>114</v>
-      </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
+    <row r="1" spans="1:14" ht="52.35" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
       <c r="I1" s="5"/>
       <c r="J1" s="5"/>
       <c r="K1" s="5"/>
@@ -1266,24 +1280,25 @@
       <c r="N1" s="5"/>
     </row>
     <row r="3" spans="1:14" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="25" t="s">
-        <v>2</v>
-      </c>
-      <c r="D3" s="26"/>
-      <c r="E3" s="26"/>
-      <c r="F3" s="26"/>
-      <c r="G3" s="26"/>
-      <c r="H3" s="27"/>
-    </row>
-    <row r="4" spans="1:14" ht="22.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="23"/>
-      <c r="B4" s="23"/>
+      <c r="C3" s="27" t="s">
+        <v>115</v>
+      </c>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="28"/>
+      <c r="G3" s="28"/>
+      <c r="H3" s="29"/>
+      <c r="I3" s="30"/>
+    </row>
+    <row r="4" spans="1:14" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="24"/>
+      <c r="B4" s="24"/>
       <c r="C4" s="7">
         <v>2019</v>
       </c>
@@ -1302,13 +1317,16 @@
       <c r="H4" s="7">
         <v>2024</v>
       </c>
+      <c r="I4" s="7">
+        <v>2025</v>
+      </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="17" t="s">
         <v>3</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>4</v>
       </c>
       <c r="C5" s="12">
         <v>5977</v>
@@ -1328,13 +1346,16 @@
       <c r="H5" s="12">
         <v>7415</v>
       </c>
+      <c r="I5" s="12">
+        <v>7854</v>
+      </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="8" t="s">
         <v>5</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>6</v>
       </c>
       <c r="C6" s="12">
         <v>5208</v>
@@ -1354,13 +1375,16 @@
       <c r="H6" s="12">
         <v>7307</v>
       </c>
+      <c r="I6" s="12">
+        <v>7042</v>
+      </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C7" s="12">
         <v>18515</v>
@@ -1378,15 +1402,18 @@
         <v>22939</v>
       </c>
       <c r="H7" s="12" t="s">
-        <v>102</v>
+        <v>101</v>
+      </c>
+      <c r="I7" s="12">
+        <v>22767</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C8" s="12">
         <v>51703</v>
@@ -1406,13 +1433,16 @@
       <c r="H8" s="12">
         <v>86446</v>
       </c>
+      <c r="I8" s="12">
+        <v>90248</v>
+      </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C9" s="12">
         <v>17835</v>
@@ -1432,13 +1462,16 @@
       <c r="H9" s="12">
         <v>33771</v>
       </c>
+      <c r="I9" s="12">
+        <v>36644</v>
+      </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C10" s="12">
         <v>6141</v>
@@ -1458,13 +1491,16 @@
       <c r="H10" s="12">
         <v>6539</v>
       </c>
+      <c r="I10" s="12">
+        <v>6449</v>
+      </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="8" t="s">
         <v>11</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>12</v>
       </c>
       <c r="C11" s="12">
         <v>429648</v>
@@ -1484,13 +1520,16 @@
       <c r="H11" s="12">
         <v>620940</v>
       </c>
+      <c r="I11" s="12">
+        <v>663366</v>
+      </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C12" s="12">
         <v>16462</v>
@@ -1510,13 +1549,16 @@
       <c r="H12" s="12">
         <v>29111</v>
       </c>
+      <c r="I12" s="12">
+        <v>26180</v>
+      </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C13" s="12">
         <v>3910</v>
@@ -1531,18 +1573,21 @@
         <v>2903</v>
       </c>
       <c r="G13" s="12" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H13" s="12">
         <v>5377</v>
       </c>
+      <c r="I13" s="12">
+        <v>5322</v>
+      </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C14" s="12">
         <v>7658</v>
@@ -1562,13 +1607,16 @@
       <c r="H14" s="12">
         <v>12239</v>
       </c>
+      <c r="I14" s="12">
+        <v>12581</v>
+      </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C15" s="12">
         <v>65516</v>
@@ -1588,13 +1636,16 @@
       <c r="H15" s="12">
         <v>89420</v>
       </c>
+      <c r="I15" s="12">
+        <v>87714</v>
+      </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C16" s="12">
         <v>7778</v>
@@ -1614,13 +1665,16 @@
       <c r="H16" s="12">
         <v>8552</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I16" s="12">
+        <v>9328</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C17" s="12">
         <v>219460</v>
@@ -1640,13 +1694,16 @@
       <c r="H17" s="12">
         <v>325509</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I17" s="12">
+        <v>341282</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18" s="8" t="s">
         <v>19</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>20</v>
       </c>
       <c r="C18" s="12">
         <v>13532</v>
@@ -1666,13 +1723,16 @@
       <c r="H18" s="12">
         <v>18158</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I18" s="12">
+        <v>18752</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C19" s="12">
         <v>3609</v>
@@ -1684,7 +1744,7 @@
         <v>1530</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G19" s="12">
         <v>1428</v>
@@ -1692,13 +1752,16 @@
       <c r="H19" s="12">
         <v>1552</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I19" s="12">
+        <v>1673</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C20" s="12">
         <v>9473</v>
@@ -1718,13 +1781,16 @@
       <c r="H20" s="12">
         <v>12238</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I20" s="12">
+        <v>12749</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C21" s="12">
         <v>2161</v>
@@ -1744,13 +1810,16 @@
       <c r="H21" s="12">
         <v>4471</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I21" s="12">
+        <v>4551</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B22" s="8" t="s">
         <v>24</v>
-      </c>
-      <c r="B22" s="8" t="s">
-        <v>25</v>
       </c>
       <c r="C22" s="12">
         <v>34183</v>
@@ -1770,13 +1839,16 @@
       <c r="H22" s="12">
         <v>45715</v>
       </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I22" s="12">
+        <v>45172</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C23" s="12">
         <v>2785</v>
@@ -1796,13 +1868,16 @@
       <c r="H23" s="12">
         <v>3987</v>
       </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I23" s="12">
+        <v>4271</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C24" s="12">
         <v>15000</v>
@@ -1822,13 +1897,16 @@
       <c r="H24" s="12">
         <v>24438</v>
       </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I24" s="12">
+        <v>24241</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C25" s="12">
         <v>31349</v>
@@ -1848,13 +1926,16 @@
       <c r="H25" s="12">
         <v>57117</v>
       </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I25" s="12">
+        <v>59534</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" s="8" t="s">
         <v>29</v>
-      </c>
-      <c r="B26" s="8" t="s">
-        <v>30</v>
       </c>
       <c r="C26" s="12">
         <v>12584</v>
@@ -1874,13 +1955,16 @@
       <c r="H26" s="12">
         <v>18115</v>
       </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I26" s="12">
+        <v>19090</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C27" s="12">
         <v>6435</v>
@@ -1900,13 +1984,16 @@
       <c r="H27" s="12">
         <v>7904</v>
       </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I27" s="12">
+        <v>9257</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C28" s="12">
         <v>35871</v>
@@ -1926,13 +2013,16 @@
       <c r="H28" s="12">
         <v>45580</v>
       </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I28" s="12">
+        <v>50963</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C29" s="12">
         <v>58731</v>
@@ -1952,13 +2042,16 @@
       <c r="H29" s="12">
         <v>95026</v>
       </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I29" s="12">
+        <v>101466</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C30" s="12">
         <v>18951</v>
@@ -1978,13 +2071,16 @@
       <c r="H30" s="12">
         <v>25122</v>
       </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I30" s="12">
+        <v>24281</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B31" s="8" t="s">
         <v>35</v>
-      </c>
-      <c r="B31" s="8" t="s">
-        <v>36</v>
       </c>
       <c r="C31" s="12">
         <v>12466</v>
@@ -2004,13 +2100,16 @@
       <c r="H31" s="12">
         <v>15424</v>
       </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I31" s="12">
+        <v>15067</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C32" s="12">
         <v>6642</v>
@@ -2030,13 +2129,16 @@
       <c r="H32" s="12">
         <v>10384</v>
       </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I32" s="12">
+        <v>9965</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C33" s="12">
         <v>29771</v>
@@ -2056,13 +2158,16 @@
       <c r="H33" s="12">
         <v>48758</v>
       </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I33" s="12">
+        <v>54054</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A34" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C34" s="12">
         <v>2367</v>
@@ -2082,13 +2187,16 @@
       <c r="H34" s="12">
         <v>4428</v>
       </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I34" s="12">
+        <v>4729</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C35" s="12">
         <v>8681</v>
@@ -2108,13 +2216,16 @@
       <c r="H35" s="12">
         <v>12060</v>
       </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I35" s="12">
+        <v>11966</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B36" s="8" t="s">
         <v>41</v>
-      </c>
-      <c r="B36" s="8" t="s">
-        <v>42</v>
       </c>
       <c r="C36" s="12">
         <v>323650</v>
@@ -2134,13 +2245,16 @@
       <c r="H36" s="12">
         <v>576448</v>
       </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I36" s="12">
+        <v>614382</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C37" s="12">
         <v>197924</v>
@@ -2160,13 +2274,16 @@
       <c r="H37" s="12">
         <v>345564</v>
       </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I37" s="12">
+        <v>364842</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C38" s="12">
         <v>2319</v>
@@ -2186,13 +2303,16 @@
       <c r="H38" s="12">
         <v>3838</v>
       </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I38" s="12">
+        <v>3896</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C39" s="12">
         <v>66439</v>
@@ -2212,13 +2332,16 @@
       <c r="H39" s="12">
         <v>109407</v>
       </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I39" s="12">
+        <v>112846</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C40" s="12">
         <v>36190</v>
@@ -2238,13 +2361,16 @@
       <c r="H40" s="12">
         <v>57399</v>
       </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I40" s="12">
+        <v>61356</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A41" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B41" s="8" t="s">
         <v>47</v>
-      </c>
-      <c r="B41" s="8" t="s">
-        <v>48</v>
       </c>
       <c r="C41" s="12">
         <v>27232</v>
@@ -2264,13 +2390,16 @@
       <c r="H41" s="12">
         <v>39299</v>
       </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I41" s="12">
+        <v>39894</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A42" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C42" s="12">
         <v>11669</v>
@@ -2290,13 +2419,16 @@
       <c r="H42" s="12">
         <v>17630</v>
       </c>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I42" s="12">
+        <v>19028</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A43" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C43" s="12">
         <v>28774</v>
@@ -2316,13 +2448,16 @@
       <c r="H43" s="12">
         <v>37957</v>
       </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I43" s="12">
+        <v>44500</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A44" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B44" s="8" t="s">
         <v>51</v>
-      </c>
-      <c r="B44" s="8" t="s">
-        <v>52</v>
       </c>
       <c r="C44" s="12">
         <v>6965</v>
@@ -2342,13 +2477,16 @@
       <c r="H44" s="12">
         <v>11317</v>
       </c>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I44" s="12">
+        <v>12185</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A45" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B45" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C45" s="12">
         <v>36663</v>
@@ -2368,13 +2506,16 @@
       <c r="H45" s="12">
         <v>47824</v>
       </c>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I45" s="12">
+        <v>48856</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A46" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B46" s="8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C46" s="12">
         <v>16311</v>
@@ -2394,13 +2535,16 @@
       <c r="H46" s="12">
         <v>34548</v>
       </c>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I46" s="12">
+        <v>34895</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A47" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C47" s="12">
         <v>22413</v>
@@ -2420,13 +2564,16 @@
       <c r="H47" s="12">
         <v>41482</v>
       </c>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I47" s="12">
+        <v>42744</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A48" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B48" s="8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C48" s="12">
         <v>42906</v>
@@ -2446,13 +2593,16 @@
       <c r="H48" s="12">
         <v>64704</v>
       </c>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I48" s="12">
+        <v>69459</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A49" s="8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B49" s="8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C49" s="12">
         <v>1674803</v>
@@ -2472,22 +2622,25 @@
       <c r="H49" s="12">
         <v>2871918</v>
       </c>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I49" s="12">
+        <v>2916965</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A50" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="B50" s="8" t="s">
         <v>58</v>
-      </c>
-      <c r="B50" s="8" t="s">
-        <v>59</v>
       </c>
       <c r="C50" s="12">
         <v>20349</v>
       </c>
       <c r="D50" s="12" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E50" s="12" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F50" s="12">
         <v>21040</v>
@@ -2498,13 +2651,16 @@
       <c r="H50" s="12">
         <v>34902</v>
       </c>
-    </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I50" s="12">
+        <v>37701</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A51" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B51" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C51" s="12">
         <v>2332</v>
@@ -2524,13 +2680,16 @@
       <c r="H51" s="12">
         <v>3869</v>
       </c>
-    </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I51" s="12">
+        <v>4115</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A52" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B52" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C52" s="12">
         <v>5134</v>
@@ -2539,24 +2698,27 @@
         <v>3474</v>
       </c>
       <c r="E52" s="12" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F52" s="12">
         <v>7282</v>
       </c>
       <c r="G52" s="12" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H52" s="12">
         <v>14614</v>
       </c>
-    </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I52" s="12">
+        <v>15622</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A53" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B53" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C53" s="12">
         <v>45920</v>
@@ -2576,13 +2738,16 @@
       <c r="H53" s="12">
         <v>68562</v>
       </c>
-    </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I53" s="12">
+        <v>70846</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A54" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B54" s="8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C54" s="12">
         <v>9692</v>
@@ -2602,13 +2767,16 @@
       <c r="H54" s="12">
         <v>15666</v>
       </c>
-    </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I54" s="12">
+        <v>13816</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A55" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="B55" s="8" t="s">
         <v>64</v>
-      </c>
-      <c r="B55" s="8" t="s">
-        <v>65</v>
       </c>
       <c r="C55" s="12">
         <v>10160</v>
@@ -2628,13 +2796,16 @@
       <c r="H55" s="12">
         <v>19241</v>
       </c>
-    </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I55" s="12">
+        <v>17769</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A56" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B56" s="8" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C56" s="12">
         <v>5758</v>
@@ -2654,13 +2825,16 @@
       <c r="H56" s="12">
         <v>8007</v>
       </c>
-    </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I56" s="12">
+        <v>8793</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A57" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B57" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C57" s="12">
         <v>370193</v>
@@ -2680,13 +2854,16 @@
       <c r="H57" s="12">
         <v>492378</v>
       </c>
-    </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I57" s="12">
+        <v>407457</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A58" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B58" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C58" s="12">
         <v>11722</v>
@@ -2706,13 +2883,16 @@
       <c r="H58" s="12">
         <v>24482</v>
       </c>
-    </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I58" s="12">
+        <v>26909</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A59" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B59" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C59" s="12">
         <v>24985</v>
@@ -2732,13 +2912,16 @@
       <c r="H59" s="12">
         <v>37082</v>
       </c>
-    </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I59" s="12">
+        <v>36132</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A60" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B60" s="8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C60" s="12">
         <v>3011</v>
@@ -2758,13 +2941,16 @@
       <c r="H60" s="12">
         <v>6758</v>
       </c>
-    </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I60" s="12">
+        <v>6972</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A61" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B61" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C61" s="12">
         <v>324232</v>
@@ -2784,13 +2970,16 @@
       <c r="H61" s="12">
         <v>496001</v>
       </c>
-    </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I61" s="12">
+        <v>525654</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A62" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B62" s="8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C62" s="12">
         <v>31334</v>
@@ -2810,13 +2999,16 @@
       <c r="H62" s="12">
         <v>65161</v>
       </c>
-    </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I62" s="12">
+        <v>68897</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A63" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B63" s="8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C63" s="12">
         <v>261827</v>
@@ -2836,13 +3028,16 @@
       <c r="H63" s="12">
         <v>314077</v>
       </c>
-    </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I63" s="12">
+        <v>312530</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A64" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B64" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C64" s="12">
         <v>54170</v>
@@ -2862,13 +3057,16 @@
       <c r="H64" s="12">
         <v>85726</v>
       </c>
+      <c r="I64" s="12">
+        <v>90226</v>
+      </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A65" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B65" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C65" s="12">
         <v>49124</v>
@@ -2888,13 +3086,16 @@
       <c r="H65" s="12">
         <v>92801</v>
       </c>
+      <c r="I65" s="12">
+        <v>90113</v>
+      </c>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A66" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B66" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C66" s="12">
         <v>814992</v>
@@ -2914,13 +3115,16 @@
       <c r="H66" s="12">
         <v>1347443</v>
       </c>
+      <c r="I66" s="12">
+        <v>1433342</v>
+      </c>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A67" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B67" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C67" s="12">
         <v>7196</v>
@@ -2940,13 +3144,16 @@
       <c r="H67" s="12">
         <v>13398</v>
       </c>
+      <c r="I67" s="12">
+        <v>12945</v>
+      </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A68" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B68" s="8" t="s">
         <v>78</v>
-      </c>
-      <c r="B68" s="8" t="s">
-        <v>79</v>
       </c>
       <c r="C68" s="12">
         <v>588631</v>
@@ -2966,13 +3173,16 @@
       <c r="H68" s="12">
         <v>987466</v>
       </c>
+      <c r="I68" s="12">
+        <v>1052541</v>
+      </c>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A69" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B69" s="8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C69" s="12">
         <v>224783</v>
@@ -2992,13 +3202,16 @@
       <c r="H69" s="12">
         <v>378043</v>
       </c>
+      <c r="I69" s="12">
+        <v>393976</v>
+      </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A70" s="8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B70" s="8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C70" s="12">
         <v>246731</v>
@@ -3018,13 +3231,16 @@
       <c r="H70" s="12">
         <v>374827</v>
       </c>
+      <c r="I70" s="12">
+        <v>391405</v>
+      </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A71" s="9" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B71" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C71" s="12">
         <v>348904</v>
@@ -3044,12 +3260,15 @@
       <c r="H71" s="12">
         <v>544219</v>
       </c>
-    </row>
-    <row r="72" spans="1:10" ht="27.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="24" t="s">
-        <v>83</v>
-      </c>
-      <c r="B72" s="24"/>
+      <c r="I71" s="12">
+        <v>573987</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10" ht="27.15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="25" t="s">
+        <v>82</v>
+      </c>
+      <c r="B72" s="25"/>
       <c r="C72" s="13">
         <v>7115840</v>
       </c>
@@ -3067,6 +3286,9 @@
       </c>
       <c r="H72" s="13">
         <v>11388355</v>
+      </c>
+      <c r="I72" s="13">
+        <v>11766152</v>
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.3">
@@ -3077,61 +3299,61 @@
       <c r="G73" s="14"/>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A74" s="21" t="s">
-        <v>93</v>
-      </c>
-      <c r="B74" s="21"/>
+      <c r="A74" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="B74" s="22"/>
     </row>
     <row r="75" spans="1:10" s="6" customFormat="1" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="28" t="s">
-        <v>115</v>
-      </c>
-      <c r="B75" s="28"/>
-      <c r="C75" s="28"/>
-      <c r="D75" s="28"/>
-      <c r="E75" s="28"/>
-      <c r="F75" s="28"/>
-      <c r="G75" s="28"/>
-      <c r="H75" s="28"/>
+      <c r="A75" s="26" t="s">
+        <v>114</v>
+      </c>
+      <c r="B75" s="26"/>
+      <c r="C75" s="26"/>
+      <c r="D75" s="26"/>
+      <c r="E75" s="26"/>
+      <c r="F75" s="26"/>
+      <c r="G75" s="26"/>
+      <c r="H75" s="26"/>
       <c r="I75" s="4"/>
       <c r="J75" s="4"/>
     </row>
-    <row r="76" spans="1:10" s="6" customFormat="1" ht="27.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="28"/>
-      <c r="B76" s="28"/>
-      <c r="C76" s="28"/>
-      <c r="D76" s="28"/>
-      <c r="E76" s="28"/>
-      <c r="F76" s="28"/>
-      <c r="G76" s="28"/>
-      <c r="H76" s="28"/>
+    <row r="76" spans="1:10" s="6" customFormat="1" ht="27.15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="26"/>
+      <c r="B76" s="26"/>
+      <c r="C76" s="26"/>
+      <c r="D76" s="26"/>
+      <c r="E76" s="26"/>
+      <c r="F76" s="26"/>
+      <c r="G76" s="26"/>
+      <c r="H76" s="26"/>
       <c r="I76" s="4"/>
       <c r="J76" s="4"/>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A77" s="20" t="s">
-        <v>104</v>
-      </c>
-      <c r="B77" s="20"/>
-      <c r="C77" s="20"/>
-      <c r="D77" s="20"/>
-      <c r="E77" s="20"/>
-      <c r="F77" s="20"/>
-      <c r="G77" s="20"/>
+      <c r="A77" s="21" t="s">
+        <v>103</v>
+      </c>
+      <c r="B77" s="21"/>
+      <c r="C77" s="21"/>
+      <c r="D77" s="21"/>
+      <c r="E77" s="21"/>
+      <c r="F77" s="21"/>
+      <c r="G77" s="21"/>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A78" s="19" t="s">
-        <v>103</v>
-      </c>
-      <c r="B78" s="20"/>
-      <c r="C78" s="20"/>
-      <c r="D78" s="20"/>
-      <c r="E78" s="20"/>
-      <c r="F78" s="20"/>
-      <c r="G78" s="20"/>
-      <c r="H78" s="20"/>
-      <c r="I78" s="20"/>
-      <c r="J78" s="20"/>
+      <c r="A78" s="20" t="s">
+        <v>102</v>
+      </c>
+      <c r="B78" s="21"/>
+      <c r="C78" s="21"/>
+      <c r="D78" s="21"/>
+      <c r="E78" s="21"/>
+      <c r="F78" s="21"/>
+      <c r="G78" s="21"/>
+      <c r="H78" s="21"/>
+      <c r="I78" s="21"/>
+      <c r="J78" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -3142,8 +3364,8 @@
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="A72:B72"/>
-    <mergeCell ref="C3:H3"/>
     <mergeCell ref="A75:H76"/>
+    <mergeCell ref="C3:I3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -3156,184 +3378,184 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AD78"/>
-  <sheetFormatPr defaultRowHeight="15.05" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28.6640625" customWidth="1"/>
     <col min="2" max="2" width="17.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="30" width="12.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" ht="52.3" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:30" ht="52.35" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="15"/>
       <c r="B1" s="5"/>
-      <c r="C1" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-      <c r="N1" s="18"/>
-      <c r="O1" s="18"/>
-      <c r="P1" s="18"/>
-      <c r="Q1" s="18"/>
-      <c r="R1" s="18"/>
-      <c r="S1" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="T1" s="18"/>
-      <c r="U1" s="18"/>
-      <c r="V1" s="18"/>
-      <c r="W1" s="18"/>
-      <c r="X1" s="18"/>
-      <c r="Y1" s="18"/>
-      <c r="Z1" s="18"/>
-      <c r="AA1" s="18"/>
-      <c r="AB1" s="18"/>
-      <c r="AC1" s="18"/>
-      <c r="AD1" s="18"/>
-    </row>
-    <row r="2" spans="1:30" ht="9.6999999999999993" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="1:30" ht="23.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="32" t="s">
+      <c r="C1" s="19" t="s">
+        <v>113</v>
+      </c>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
+      <c r="N1" s="19"/>
+      <c r="O1" s="19"/>
+      <c r="P1" s="19"/>
+      <c r="Q1" s="19"/>
+      <c r="R1" s="19"/>
+      <c r="S1" s="19" t="s">
+        <v>113</v>
+      </c>
+      <c r="T1" s="19"/>
+      <c r="U1" s="19"/>
+      <c r="V1" s="19"/>
+      <c r="W1" s="19"/>
+      <c r="X1" s="19"/>
+      <c r="Y1" s="19"/>
+      <c r="Z1" s="19"/>
+      <c r="AA1" s="19"/>
+      <c r="AB1" s="19"/>
+      <c r="AC1" s="19"/>
+      <c r="AD1" s="19"/>
+    </row>
+    <row r="2" spans="1:30" ht="9.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="1:30" ht="23.7" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="32" t="s">
+      <c r="B3" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="29" t="s">
+      <c r="C3" s="31" t="s">
+        <v>115</v>
+      </c>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
+      <c r="G3" s="32"/>
+      <c r="H3" s="32"/>
+      <c r="I3" s="32"/>
+      <c r="J3" s="32"/>
+      <c r="K3" s="32"/>
+      <c r="L3" s="32"/>
+      <c r="M3" s="32"/>
+      <c r="N3" s="32"/>
+      <c r="O3" s="32"/>
+      <c r="P3" s="32"/>
+      <c r="Q3" s="32"/>
+      <c r="R3" s="33"/>
+      <c r="S3" s="31" t="s">
+        <v>115</v>
+      </c>
+      <c r="T3" s="32"/>
+      <c r="U3" s="32"/>
+      <c r="V3" s="32"/>
+      <c r="W3" s="32"/>
+      <c r="X3" s="32"/>
+      <c r="Y3" s="32"/>
+      <c r="Z3" s="32"/>
+      <c r="AA3" s="32"/>
+      <c r="AB3" s="32"/>
+      <c r="AC3" s="32"/>
+      <c r="AD3" s="33"/>
+    </row>
+    <row r="4" spans="1:30" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="35"/>
+      <c r="B4" s="35"/>
+      <c r="C4" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="N4" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="O4" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="P4" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="Q4" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="R4" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="S4" s="16" t="s">
+        <v>104</v>
+      </c>
+      <c r="T4" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="U4" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="V4" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="W4" s="16" t="s">
+        <v>108</v>
+      </c>
+      <c r="X4" s="16" t="s">
+        <v>109</v>
+      </c>
+      <c r="Y4" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z4" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="AA4" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="AB4" s="16" t="s">
         <v>116</v>
       </c>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="30"/>
-      <c r="G3" s="30"/>
-      <c r="H3" s="30"/>
-      <c r="I3" s="30"/>
-      <c r="J3" s="30"/>
-      <c r="K3" s="30"/>
-      <c r="L3" s="30"/>
-      <c r="M3" s="30"/>
-      <c r="N3" s="30"/>
-      <c r="O3" s="30"/>
-      <c r="P3" s="30"/>
-      <c r="Q3" s="30"/>
-      <c r="R3" s="31"/>
-      <c r="S3" s="29" t="s">
-        <v>116</v>
-      </c>
-      <c r="T3" s="30"/>
-      <c r="U3" s="30"/>
-      <c r="V3" s="30"/>
-      <c r="W3" s="30"/>
-      <c r="X3" s="30"/>
-      <c r="Y3" s="30"/>
-      <c r="Z3" s="30"/>
-      <c r="AA3" s="30"/>
-      <c r="AB3" s="30"/>
-      <c r="AC3" s="30"/>
-      <c r="AD3" s="31"/>
-    </row>
-    <row r="4" spans="1:30" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="33"/>
-      <c r="B4" s="33"/>
-      <c r="C4" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="M4" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="N4" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="O4" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="P4" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="Q4" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="R4" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="S4" s="16" t="s">
-        <v>105</v>
-      </c>
-      <c r="T4" s="16" t="s">
-        <v>106</v>
-      </c>
-      <c r="U4" s="16" t="s">
-        <v>107</v>
-      </c>
-      <c r="V4" s="16" t="s">
-        <v>108</v>
-      </c>
-      <c r="W4" s="16" t="s">
-        <v>109</v>
-      </c>
-      <c r="X4" s="16" t="s">
-        <v>110</v>
-      </c>
-      <c r="Y4" s="16" t="s">
-        <v>111</v>
-      </c>
-      <c r="Z4" s="16" t="s">
-        <v>112</v>
-      </c>
-      <c r="AA4" s="16" t="s">
-        <v>113</v>
-      </c>
-      <c r="AB4" s="16" t="s">
+      <c r="AC4" s="16" t="s">
         <v>117</v>
       </c>
-      <c r="AC4" s="16" t="s">
+      <c r="AD4" s="16" t="s">
         <v>118</v>
-      </c>
-      <c r="AD4" s="16" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="5" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>3</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>4</v>
       </c>
       <c r="C5" s="10">
         <v>920</v>
@@ -3413,15 +3635,19 @@
       <c r="AB5" s="10">
         <v>1725</v>
       </c>
-      <c r="AC5" s="10"/>
-      <c r="AD5" s="10"/>
+      <c r="AC5" s="10">
+        <v>2812</v>
+      </c>
+      <c r="AD5" s="10">
+        <v>1969</v>
+      </c>
     </row>
     <row r="6" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>6</v>
       </c>
       <c r="C6" s="10">
         <v>1066</v>
@@ -3475,10 +3701,10 @@
         <v>1136</v>
       </c>
       <c r="T6" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="U6" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="V6" s="10">
         <v>1541</v>
@@ -3501,15 +3727,19 @@
       <c r="AB6" s="10">
         <v>1391</v>
       </c>
-      <c r="AC6" s="10"/>
-      <c r="AD6" s="10"/>
+      <c r="AC6" s="10">
+        <v>2459</v>
+      </c>
+      <c r="AD6" s="10">
+        <v>1852</v>
+      </c>
     </row>
     <row r="7" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C7" s="10">
         <v>2319</v>
@@ -3527,7 +3757,7 @@
         <v>3356</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I7" s="10">
         <v>4934</v>
@@ -3572,16 +3802,16 @@
         <v>4455</v>
       </c>
       <c r="W7" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="X7" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="Y7" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="Z7" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="AA7" s="10">
         <v>3354</v>
@@ -3589,15 +3819,19 @@
       <c r="AB7" s="10">
         <v>5402</v>
       </c>
-      <c r="AC7" s="10"/>
-      <c r="AD7" s="10"/>
+      <c r="AC7" s="10">
+        <v>9410</v>
+      </c>
+      <c r="AD7" s="10">
+        <v>4601</v>
+      </c>
     </row>
     <row r="8" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C8" s="10">
         <v>511</v>
@@ -3636,7 +3870,7 @@
         <v>2003</v>
       </c>
       <c r="O8" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="P8" s="10">
         <v>11084</v>
@@ -3648,7 +3882,7 @@
         <v>2286</v>
       </c>
       <c r="S8" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="T8" s="10">
         <v>14095</v>
@@ -3660,7 +3894,7 @@
         <v>2590</v>
       </c>
       <c r="W8" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="X8" s="10">
         <v>16270</v>
@@ -3669,7 +3903,7 @@
         <v>65149</v>
       </c>
       <c r="Z8" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="AA8" s="10">
         <v>1145</v>
@@ -3677,15 +3911,19 @@
       <c r="AB8" s="10">
         <v>16417</v>
       </c>
-      <c r="AC8" s="10"/>
-      <c r="AD8" s="10"/>
+      <c r="AC8" s="10">
+        <v>68325</v>
+      </c>
+      <c r="AD8" s="10">
+        <v>4362</v>
+      </c>
     </row>
     <row r="9" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C9" s="10">
         <v>1027</v>
@@ -3765,15 +4003,19 @@
       <c r="AB9" s="10">
         <v>8131</v>
       </c>
-      <c r="AC9" s="10"/>
-      <c r="AD9" s="10"/>
+      <c r="AC9" s="10">
+        <v>20884</v>
+      </c>
+      <c r="AD9" s="10">
+        <v>5457</v>
+      </c>
     </row>
     <row r="10" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C10" s="10">
         <v>1192</v>
@@ -3853,15 +4095,19 @@
       <c r="AB10" s="10">
         <v>1519</v>
       </c>
-      <c r="AC10" s="10"/>
-      <c r="AD10" s="10"/>
+      <c r="AC10" s="10">
+        <v>2554</v>
+      </c>
+      <c r="AD10" s="10">
+        <v>1237</v>
+      </c>
     </row>
     <row r="11" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>11</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>12</v>
       </c>
       <c r="C11" s="10">
         <v>23140</v>
@@ -3941,15 +4187,19 @@
       <c r="AB11" s="10">
         <v>171685</v>
       </c>
-      <c r="AC11" s="10"/>
-      <c r="AD11" s="10"/>
+      <c r="AC11" s="10">
+        <v>355877</v>
+      </c>
+      <c r="AD11" s="10">
+        <v>100491</v>
+      </c>
     </row>
     <row r="12" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C12" s="10">
         <v>971</v>
@@ -3967,13 +4217,13 @@
         <v>1162</v>
       </c>
       <c r="H12" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="J12" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="K12" s="10">
         <v>397</v>
@@ -4021,7 +4271,7 @@
         <v>13372</v>
       </c>
       <c r="Z12" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="AA12" s="10">
         <v>1323</v>
@@ -4029,15 +4279,19 @@
       <c r="AB12" s="10">
         <v>5530</v>
       </c>
-      <c r="AC12" s="10"/>
-      <c r="AD12" s="10"/>
+      <c r="AC12" s="10">
+        <v>14823</v>
+      </c>
+      <c r="AD12" s="10">
+        <v>4504</v>
+      </c>
     </row>
     <row r="13" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C13" s="10">
         <v>645</v>
@@ -4067,10 +4321,10 @@
         <v>383</v>
       </c>
       <c r="L13" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M13" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="N13" s="10">
         <v>783</v>
@@ -4100,7 +4354,7 @@
         <v>1541</v>
       </c>
       <c r="W13" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="X13" s="10">
         <v>1099</v>
@@ -4117,15 +4371,19 @@
       <c r="AB13" s="10">
         <v>1457</v>
       </c>
-      <c r="AC13" s="10"/>
-      <c r="AD13" s="10"/>
+      <c r="AC13" s="10">
+        <v>1189</v>
+      </c>
+      <c r="AD13" s="10">
+        <v>1603</v>
+      </c>
     </row>
     <row r="14" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C14" s="10">
         <v>1827</v>
@@ -4146,7 +4404,7 @@
         <v>1164</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="J14" s="10">
         <v>1417</v>
@@ -4155,7 +4413,7 @@
         <v>612</v>
       </c>
       <c r="L14" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M14" s="10">
         <v>2828</v>
@@ -4194,7 +4452,7 @@
         <v>2257</v>
       </c>
       <c r="Y14" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="Z14" s="10">
         <v>3264</v>
@@ -4205,15 +4463,19 @@
       <c r="AB14" s="10">
         <v>2175</v>
       </c>
-      <c r="AC14" s="10"/>
-      <c r="AD14" s="10"/>
+      <c r="AC14" s="10">
+        <v>4589</v>
+      </c>
+      <c r="AD14" s="10">
+        <v>3347</v>
+      </c>
     </row>
     <row r="15" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C15" s="10">
         <v>2717</v>
@@ -4252,7 +4514,7 @@
         <v>6132</v>
       </c>
       <c r="O15" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="P15" s="10">
         <v>14356</v>
@@ -4261,7 +4523,7 @@
         <v>48753</v>
       </c>
       <c r="R15" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="S15" s="10">
         <v>2856</v>
@@ -4293,15 +4555,19 @@
       <c r="AB15" s="10">
         <v>20635</v>
       </c>
-      <c r="AC15" s="10"/>
-      <c r="AD15" s="10"/>
+      <c r="AC15" s="10">
+        <v>55194</v>
+      </c>
+      <c r="AD15" s="10">
+        <v>9013</v>
+      </c>
     </row>
     <row r="16" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C16" s="10">
         <v>1556</v>
@@ -4346,7 +4612,7 @@
         <v>1283</v>
       </c>
       <c r="Q16" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="R16" s="10">
         <v>1474</v>
@@ -4381,15 +4647,19 @@
       <c r="AB16" s="10">
         <v>2205</v>
       </c>
-      <c r="AC16" s="10"/>
-      <c r="AD16" s="10"/>
+      <c r="AC16" s="10">
+        <v>3298</v>
+      </c>
+      <c r="AD16" s="10">
+        <v>2140</v>
+      </c>
     </row>
     <row r="17" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C17" s="10">
         <v>3751</v>
@@ -4416,7 +4686,7 @@
         <v>6603</v>
       </c>
       <c r="K17" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="L17" s="10">
         <v>19539</v>
@@ -4469,15 +4739,19 @@
       <c r="AB17" s="10">
         <v>71929</v>
       </c>
-      <c r="AC17" s="10"/>
-      <c r="AD17" s="10"/>
+      <c r="AC17" s="10">
+        <v>238220</v>
+      </c>
+      <c r="AD17" s="10">
+        <v>25733</v>
+      </c>
     </row>
     <row r="18" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>20</v>
       </c>
       <c r="C18" s="10">
         <v>1389</v>
@@ -4531,7 +4805,7 @@
         <v>1798</v>
       </c>
       <c r="T18" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="U18" s="10">
         <v>9258</v>
@@ -4557,15 +4831,19 @@
       <c r="AB18" s="10">
         <v>4396</v>
       </c>
-      <c r="AC18" s="10"/>
-      <c r="AD18" s="10"/>
+      <c r="AC18" s="10">
+        <v>9919</v>
+      </c>
+      <c r="AD18" s="10">
+        <v>2383</v>
+      </c>
     </row>
     <row r="19" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C19" s="10">
         <v>609</v>
@@ -4645,15 +4923,19 @@
       <c r="AB19" s="10">
         <v>351</v>
       </c>
-      <c r="AC19" s="10"/>
-      <c r="AD19" s="10"/>
+      <c r="AC19" s="10">
+        <v>562</v>
+      </c>
+      <c r="AD19" s="10">
+        <v>373</v>
+      </c>
     </row>
     <row r="20" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C20" s="10">
         <v>1496</v>
@@ -4733,15 +5015,19 @@
       <c r="AB20" s="10">
         <v>2975</v>
       </c>
-      <c r="AC20" s="10"/>
-      <c r="AD20" s="10"/>
+      <c r="AC20" s="10">
+        <v>5692</v>
+      </c>
+      <c r="AD20" s="10">
+        <v>2307</v>
+      </c>
     </row>
     <row r="21" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C21" s="10">
         <v>467</v>
@@ -4821,15 +5107,19 @@
       <c r="AB21" s="10">
         <v>1005</v>
       </c>
-      <c r="AC21" s="10"/>
-      <c r="AD21" s="10"/>
+      <c r="AC21" s="10">
+        <v>1152</v>
+      </c>
+      <c r="AD21" s="10">
+        <v>1299</v>
+      </c>
     </row>
     <row r="22" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B22" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>25</v>
       </c>
       <c r="C22" s="10">
         <v>5829</v>
@@ -4909,15 +5199,19 @@
       <c r="AB22" s="10">
         <v>10236</v>
       </c>
-      <c r="AC22" s="10"/>
-      <c r="AD22" s="10"/>
+      <c r="AC22" s="10">
+        <v>13404</v>
+      </c>
+      <c r="AD22" s="10">
+        <v>12381</v>
+      </c>
     </row>
     <row r="23" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C23" s="10">
         <v>514</v>
@@ -4997,15 +5291,19 @@
       <c r="AB23" s="10">
         <v>1030</v>
       </c>
-      <c r="AC23" s="10"/>
-      <c r="AD23" s="10"/>
+      <c r="AC23" s="10">
+        <v>1641</v>
+      </c>
+      <c r="AD23" s="10">
+        <v>931</v>
+      </c>
     </row>
     <row r="24" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C24" s="10">
         <v>690</v>
@@ -5062,7 +5360,7 @@
         <v>5380</v>
       </c>
       <c r="U24" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="V24" s="10">
         <v>2951</v>
@@ -5080,20 +5378,24 @@
         <v>3460</v>
       </c>
       <c r="AA24" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="AB24" s="10">
         <v>4953</v>
       </c>
-      <c r="AC24" s="10"/>
-      <c r="AD24" s="10"/>
+      <c r="AC24" s="10">
+        <v>14898</v>
+      </c>
+      <c r="AD24" s="10">
+        <v>2918</v>
+      </c>
     </row>
     <row r="25" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C25" s="10">
         <v>801</v>
@@ -5173,15 +5475,19 @@
       <c r="AB25" s="10">
         <v>13538</v>
       </c>
-      <c r="AC25" s="10"/>
-      <c r="AD25" s="10"/>
+      <c r="AC25" s="10">
+        <v>39583</v>
+      </c>
+      <c r="AD25" s="10">
+        <v>4998</v>
+      </c>
     </row>
     <row r="26" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>30</v>
       </c>
       <c r="C26" s="10">
         <v>2082</v>
@@ -5261,15 +5567,19 @@
       <c r="AB26" s="10">
         <v>4464</v>
       </c>
-      <c r="AC26" s="10"/>
-      <c r="AD26" s="10"/>
+      <c r="AC26" s="10">
+        <v>6902</v>
+      </c>
+      <c r="AD26" s="10">
+        <v>4457</v>
+      </c>
     </row>
     <row r="27" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C27" s="10">
         <v>1464</v>
@@ -5349,15 +5659,19 @@
       <c r="AB27" s="10">
         <v>2196</v>
       </c>
-      <c r="AC27" s="10"/>
-      <c r="AD27" s="10"/>
+      <c r="AC27" s="10">
+        <v>2241</v>
+      </c>
+      <c r="AD27" s="10">
+        <v>2565</v>
+      </c>
     </row>
     <row r="28" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C28" s="10">
         <v>4461</v>
@@ -5437,15 +5751,19 @@
       <c r="AB28" s="10">
         <v>11076</v>
       </c>
-      <c r="AC28" s="10"/>
-      <c r="AD28" s="10"/>
+      <c r="AC28" s="10">
+        <v>22959</v>
+      </c>
+      <c r="AD28" s="10">
+        <v>9615</v>
+      </c>
     </row>
     <row r="29" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C29" s="10">
         <v>548</v>
@@ -5505,7 +5823,7 @@
         <v>61889</v>
       </c>
       <c r="V29" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="W29" s="10">
         <v>1317</v>
@@ -5520,20 +5838,24 @@
         <v>5375</v>
       </c>
       <c r="AA29" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="AB29" s="10">
         <v>22154</v>
       </c>
-      <c r="AC29" s="10"/>
-      <c r="AD29" s="10"/>
+      <c r="AC29" s="10">
+        <v>71789</v>
+      </c>
+      <c r="AD29" s="10">
+        <v>5920</v>
+      </c>
     </row>
     <row r="30" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C30" s="10">
         <v>2759</v>
@@ -5613,15 +5935,19 @@
       <c r="AB30" s="10">
         <v>6917</v>
       </c>
-      <c r="AC30" s="10"/>
-      <c r="AD30" s="10"/>
+      <c r="AC30" s="10">
+        <v>6948</v>
+      </c>
+      <c r="AD30" s="10">
+        <v>6285</v>
+      </c>
     </row>
     <row r="31" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B31" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>36</v>
       </c>
       <c r="C31" s="10">
         <v>1172</v>
@@ -5701,15 +6027,19 @@
       <c r="AB31" s="10">
         <v>4004</v>
       </c>
-      <c r="AC31" s="10"/>
-      <c r="AD31" s="10"/>
+      <c r="AC31" s="10">
+        <v>6712</v>
+      </c>
+      <c r="AD31" s="10">
+        <v>2888</v>
+      </c>
     </row>
     <row r="32" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C32" s="10">
         <v>1715</v>
@@ -5763,7 +6093,7 @@
         <v>2783</v>
       </c>
       <c r="T32" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="U32" s="10">
         <v>2338</v>
@@ -5789,15 +6119,19 @@
       <c r="AB32" s="10">
         <v>2371</v>
       </c>
-      <c r="AC32" s="10"/>
-      <c r="AD32" s="10"/>
+      <c r="AC32" s="10">
+        <v>2457</v>
+      </c>
+      <c r="AD32" s="10">
+        <v>2487</v>
+      </c>
     </row>
     <row r="33" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C33" s="10">
         <v>2242</v>
@@ -5877,15 +6211,19 @@
       <c r="AB33" s="10">
         <v>12633</v>
       </c>
-      <c r="AC33" s="10"/>
-      <c r="AD33" s="10"/>
+      <c r="AC33" s="10">
+        <v>29978</v>
+      </c>
+      <c r="AD33" s="10">
+        <v>7648</v>
+      </c>
     </row>
     <row r="34" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C34" s="10">
         <v>566</v>
@@ -5965,15 +6303,19 @@
       <c r="AB34" s="10">
         <v>904</v>
       </c>
-      <c r="AC34" s="10"/>
-      <c r="AD34" s="10"/>
+      <c r="AC34" s="10">
+        <v>1435</v>
+      </c>
+      <c r="AD34" s="10">
+        <v>1260</v>
+      </c>
     </row>
     <row r="35" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C35" s="10">
         <v>1150</v>
@@ -6053,15 +6395,19 @@
       <c r="AB35" s="10">
         <v>3801</v>
       </c>
-      <c r="AC35" s="10"/>
-      <c r="AD35" s="10"/>
+      <c r="AC35" s="10">
+        <v>3916</v>
+      </c>
+      <c r="AD35" s="10">
+        <v>2525</v>
+      </c>
     </row>
     <row r="36" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B36" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>42</v>
       </c>
       <c r="C36" s="10">
         <v>3902</v>
@@ -6121,7 +6467,7 @@
         <v>324098</v>
       </c>
       <c r="V36" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="W36" s="10">
         <v>7920</v>
@@ -6141,15 +6487,19 @@
       <c r="AB36" s="10">
         <v>148820</v>
       </c>
-      <c r="AC36" s="10"/>
-      <c r="AD36" s="10"/>
+      <c r="AC36" s="10">
+        <v>379053</v>
+      </c>
+      <c r="AD36" s="10">
+        <v>76984</v>
+      </c>
     </row>
     <row r="37" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C37" s="10">
         <v>1969</v>
@@ -6188,7 +6538,7 @@
         <v>13830</v>
       </c>
       <c r="O37" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="P37" s="10">
         <v>55076</v>
@@ -6203,16 +6553,16 @@
         <v>2606</v>
       </c>
       <c r="T37" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="U37" s="10">
         <v>204418</v>
       </c>
       <c r="V37" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="W37" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="X37" s="10">
         <v>84004</v>
@@ -6229,15 +6579,19 @@
       <c r="AB37" s="10">
         <v>88481</v>
       </c>
-      <c r="AC37" s="10"/>
-      <c r="AD37" s="10"/>
+      <c r="AC37" s="10">
+        <v>239986</v>
+      </c>
+      <c r="AD37" s="10">
+        <v>32536</v>
+      </c>
     </row>
     <row r="38" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C38" s="10">
         <v>18</v>
@@ -6297,7 +6651,7 @@
         <v>2453</v>
       </c>
       <c r="V38" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="W38" s="10">
         <v>42</v>
@@ -6317,15 +6671,19 @@
       <c r="AB38" s="10">
         <v>840</v>
       </c>
-      <c r="AC38" s="10"/>
-      <c r="AD38" s="10"/>
+      <c r="AC38" s="10">
+        <v>2650</v>
+      </c>
+      <c r="AD38" s="10">
+        <v>350</v>
+      </c>
     </row>
     <row r="39" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C39" s="10">
         <v>1444</v>
@@ -6364,7 +6722,7 @@
         <v>5394</v>
       </c>
       <c r="O39" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="P39" s="10">
         <v>20729</v>
@@ -6388,7 +6746,7 @@
         <v>8060</v>
       </c>
       <c r="W39" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="X39" s="10">
         <v>25283</v>
@@ -6405,15 +6763,19 @@
       <c r="AB39" s="10">
         <v>26745</v>
       </c>
-      <c r="AC39" s="10"/>
-      <c r="AD39" s="10"/>
+      <c r="AC39" s="10">
+        <v>72775</v>
+      </c>
+      <c r="AD39" s="10">
+        <v>10057</v>
+      </c>
     </row>
     <row r="40" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C40" s="10">
         <v>490</v>
@@ -6493,15 +6855,19 @@
       <c r="AB40" s="10">
         <v>11695</v>
       </c>
-      <c r="AC40" s="10"/>
-      <c r="AD40" s="10"/>
+      <c r="AC40" s="10">
+        <v>43674</v>
+      </c>
+      <c r="AD40" s="10">
+        <v>4937</v>
+      </c>
     </row>
     <row r="41" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B41" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>48</v>
       </c>
       <c r="C41" s="10">
         <v>3050</v>
@@ -6581,15 +6947,19 @@
       <c r="AB41" s="10">
         <v>9931</v>
       </c>
-      <c r="AC41" s="10"/>
-      <c r="AD41" s="10"/>
+      <c r="AC41" s="10">
+        <v>18752</v>
+      </c>
+      <c r="AD41" s="10">
+        <v>6289</v>
+      </c>
     </row>
     <row r="42" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C42" s="10">
         <v>1697</v>
@@ -6669,15 +7039,19 @@
       <c r="AB42" s="10">
         <v>4669</v>
       </c>
-      <c r="AC42" s="10"/>
-      <c r="AD42" s="10"/>
+      <c r="AC42" s="10">
+        <v>8628</v>
+      </c>
+      <c r="AD42" s="10">
+        <v>3613</v>
+      </c>
     </row>
     <row r="43" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C43" s="10">
         <v>1162</v>
@@ -6719,16 +7093,16 @@
         <v>734</v>
       </c>
       <c r="P43" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="Q43" s="10">
         <v>15661</v>
       </c>
       <c r="R43" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="S43" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="T43" s="10">
         <v>8274</v>
@@ -6757,15 +7131,19 @@
       <c r="AB43" s="10">
         <v>10486</v>
       </c>
-      <c r="AC43" s="10"/>
-      <c r="AD43" s="10"/>
+      <c r="AC43" s="10">
+        <v>21962</v>
+      </c>
+      <c r="AD43" s="10" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="44" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B44" s="1" t="s">
         <v>51</v>
-      </c>
-      <c r="B44" s="1" t="s">
-        <v>52</v>
       </c>
       <c r="C44" s="10">
         <v>1186</v>
@@ -6845,15 +7223,19 @@
       <c r="AB44" s="10">
         <v>2623</v>
       </c>
-      <c r="AC44" s="10"/>
-      <c r="AD44" s="10"/>
+      <c r="AC44" s="10">
+        <v>4022</v>
+      </c>
+      <c r="AD44" s="10">
+        <v>3260</v>
+      </c>
     </row>
     <row r="45" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C45" s="10">
         <v>2693</v>
@@ -6889,7 +7271,7 @@
         <v>18050</v>
       </c>
       <c r="N45" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="O45" s="10">
         <v>2480</v>
@@ -6910,13 +7292,13 @@
         <v>12547</v>
       </c>
       <c r="U45" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="V45" s="10">
         <v>7263</v>
       </c>
       <c r="W45" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="X45" s="10">
         <v>13473</v>
@@ -6933,15 +7315,19 @@
       <c r="AB45" s="10">
         <v>14215</v>
       </c>
-      <c r="AC45" s="10"/>
-      <c r="AD45" s="10"/>
+      <c r="AC45" s="10">
+        <v>21877</v>
+      </c>
+      <c r="AD45" s="10">
+        <v>8386</v>
+      </c>
     </row>
     <row r="46" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C46" s="10">
         <v>1934</v>
@@ -6977,7 +7363,7 @@
         <v>7271</v>
       </c>
       <c r="N46" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="O46" s="10">
         <v>1895</v>
@@ -6995,7 +7381,7 @@
         <v>2571</v>
       </c>
       <c r="T46" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="U46" s="10">
         <v>14344</v>
@@ -7021,15 +7407,19 @@
       <c r="AB46" s="10">
         <v>8979</v>
       </c>
-      <c r="AC46" s="10"/>
-      <c r="AD46" s="10"/>
+      <c r="AC46" s="10">
+        <v>16137</v>
+      </c>
+      <c r="AD46" s="10">
+        <v>6317</v>
+      </c>
     </row>
     <row r="47" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C47" s="10">
         <v>1466</v>
@@ -7109,15 +7499,19 @@
       <c r="AB47" s="10">
         <v>10481</v>
       </c>
-      <c r="AC47" s="10"/>
-      <c r="AD47" s="10"/>
+      <c r="AC47" s="10">
+        <v>23093</v>
+      </c>
+      <c r="AD47" s="10">
+        <v>6294</v>
+      </c>
     </row>
     <row r="48" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C48" s="10">
         <v>2213</v>
@@ -7180,7 +7574,7 @@
         <v>6934</v>
       </c>
       <c r="W48" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="X48" s="10">
         <v>15289</v>
@@ -7197,15 +7591,19 @@
       <c r="AB48" s="10">
         <v>16155</v>
       </c>
-      <c r="AC48" s="10"/>
-      <c r="AD48" s="10"/>
+      <c r="AC48" s="10">
+        <v>39582</v>
+      </c>
+      <c r="AD48" s="10">
+        <v>9375</v>
+      </c>
     </row>
     <row r="49" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C49" s="10">
         <v>130184</v>
@@ -7285,15 +7683,19 @@
       <c r="AB49" s="10">
         <v>790970</v>
       </c>
-      <c r="AC49" s="10"/>
-      <c r="AD49" s="10"/>
+      <c r="AC49" s="10">
+        <v>1336327</v>
+      </c>
+      <c r="AD49" s="10">
+        <v>542842</v>
+      </c>
     </row>
     <row r="50" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B50" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="B50" s="1" t="s">
-        <v>59</v>
       </c>
       <c r="C50" s="10">
         <v>1379</v>
@@ -7308,28 +7710,28 @@
         <v>2332</v>
       </c>
       <c r="G50" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H50" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I50" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="J50" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="K50" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="L50" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M50" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="N50" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="O50" s="10">
         <v>1147</v>
@@ -7373,15 +7775,19 @@
       <c r="AB50" s="10">
         <v>8950</v>
       </c>
-      <c r="AC50" s="10"/>
-      <c r="AD50" s="10"/>
+      <c r="AC50" s="10">
+        <v>23417</v>
+      </c>
+      <c r="AD50" s="10">
+        <v>3570</v>
+      </c>
     </row>
     <row r="51" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C51" s="10">
         <v>65</v>
@@ -7435,7 +7841,7 @@
         <v>83</v>
       </c>
       <c r="T51" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="U51" s="10">
         <v>2295</v>
@@ -7461,15 +7867,19 @@
       <c r="AB51" s="10">
         <v>775</v>
       </c>
-      <c r="AC51" s="10"/>
-      <c r="AD51" s="10"/>
+      <c r="AC51" s="10">
+        <v>2813</v>
+      </c>
+      <c r="AD51" s="10" t="s">
+        <v>101</v>
+      </c>
     </row>
     <row r="52" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C52" s="10">
         <v>616</v>
@@ -7496,16 +7906,16 @@
         <v>753</v>
       </c>
       <c r="K52" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="L52" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M52" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="N52" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="O52" s="10">
         <v>320</v>
@@ -7517,16 +7927,16 @@
         <v>3846</v>
       </c>
       <c r="R52" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="S52" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="T52" s="10">
         <v>1599</v>
       </c>
       <c r="U52" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="V52" s="10">
         <v>1671</v>
@@ -7535,13 +7945,13 @@
         <v>510</v>
       </c>
       <c r="X52" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="Y52" s="10">
         <v>8767</v>
       </c>
       <c r="Z52" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="AA52" s="10">
         <v>887</v>
@@ -7549,15 +7959,19 @@
       <c r="AB52" s="10">
         <v>3157</v>
       </c>
-      <c r="AC52" s="10"/>
-      <c r="AD52" s="10"/>
+      <c r="AC52" s="10">
+        <v>9270</v>
+      </c>
+      <c r="AD52" s="10">
+        <v>2308</v>
+      </c>
     </row>
     <row r="53" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C53" s="10">
         <v>1409</v>
@@ -7590,16 +8004,16 @@
         <v>2917</v>
       </c>
       <c r="M53" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="N53" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="O53" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="P53" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="Q53" s="10">
         <v>33944</v>
@@ -7637,15 +8051,19 @@
       <c r="AB53" s="10">
         <v>16557</v>
       </c>
-      <c r="AC53" s="10"/>
-      <c r="AD53" s="10"/>
+      <c r="AC53" s="10">
+        <v>45976</v>
+      </c>
+      <c r="AD53" s="10">
+        <v>6800</v>
+      </c>
     </row>
     <row r="54" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C54" s="10">
         <v>1117</v>
@@ -7725,15 +8143,19 @@
       <c r="AB54" s="10">
         <v>2969</v>
       </c>
-      <c r="AC54" s="10"/>
-      <c r="AD54" s="10"/>
+      <c r="AC54" s="10">
+        <v>8655</v>
+      </c>
+      <c r="AD54" s="10">
+        <v>1311</v>
+      </c>
     </row>
     <row r="55" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B55" s="1" t="s">
         <v>64</v>
-      </c>
-      <c r="B55" s="1" t="s">
-        <v>65</v>
       </c>
       <c r="C55" s="10">
         <v>675</v>
@@ -7813,15 +8235,19 @@
       <c r="AB55" s="10">
         <v>4378</v>
       </c>
-      <c r="AC55" s="10"/>
-      <c r="AD55" s="10"/>
+      <c r="AC55" s="10">
+        <v>9993</v>
+      </c>
+      <c r="AD55" s="10">
+        <v>1974</v>
+      </c>
     </row>
     <row r="56" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C56" s="10">
         <v>376</v>
@@ -7860,7 +8286,7 @@
         <v>547</v>
       </c>
       <c r="O56" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="P56" s="10">
         <v>1487</v>
@@ -7896,20 +8322,24 @@
         <v>560</v>
       </c>
       <c r="AA56" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="AB56" s="10">
         <v>1887</v>
       </c>
-      <c r="AC56" s="10"/>
-      <c r="AD56" s="10"/>
+      <c r="AC56" s="10">
+        <v>5924</v>
+      </c>
+      <c r="AD56" s="10">
+        <v>587</v>
+      </c>
     </row>
     <row r="57" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C57" s="10">
         <v>7738</v>
@@ -7989,15 +8419,19 @@
       <c r="AB57" s="10">
         <v>113137</v>
       </c>
-      <c r="AC57" s="10"/>
-      <c r="AD57" s="10"/>
+      <c r="AC57" s="10">
+        <v>234069</v>
+      </c>
+      <c r="AD57" s="10">
+        <v>50819</v>
+      </c>
     </row>
     <row r="58" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C58" s="10">
         <v>275</v>
@@ -8036,7 +8470,7 @@
         <v>1343</v>
       </c>
       <c r="O58" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="P58" s="10">
         <v>2697</v>
@@ -8051,7 +8485,7 @@
         <v>450</v>
       </c>
       <c r="T58" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="U58" s="10">
         <v>15811</v>
@@ -8077,15 +8511,19 @@
       <c r="AB58" s="10">
         <v>5079</v>
       </c>
-      <c r="AC58" s="10"/>
-      <c r="AD58" s="10"/>
+      <c r="AC58" s="10">
+        <v>17932</v>
+      </c>
+      <c r="AD58" s="10">
+        <v>3088</v>
+      </c>
     </row>
     <row r="59" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C59" s="10">
         <v>404</v>
@@ -8133,7 +8571,7 @@
         <v>20715</v>
       </c>
       <c r="R59" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="S59" s="10">
         <v>657</v>
@@ -8165,15 +8603,19 @@
       <c r="AB59" s="10">
         <v>7529</v>
       </c>
-      <c r="AC59" s="10"/>
-      <c r="AD59" s="10"/>
+      <c r="AC59" s="10">
+        <v>24048</v>
+      </c>
+      <c r="AD59" s="10">
+        <v>3933</v>
+      </c>
     </row>
     <row r="60" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C60" s="10">
         <v>63</v>
@@ -8197,7 +8639,7 @@
         <v>1732</v>
       </c>
       <c r="J60" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="K60" s="10">
         <v>71</v>
@@ -8233,7 +8675,7 @@
         <v>4807</v>
       </c>
       <c r="V60" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="W60" s="10">
         <v>262</v>
@@ -8253,15 +8695,19 @@
       <c r="AB60" s="10">
         <v>1434</v>
       </c>
-      <c r="AC60" s="10"/>
-      <c r="AD60" s="10"/>
+      <c r="AC60" s="10">
+        <v>4691</v>
+      </c>
+      <c r="AD60" s="10">
+        <v>579</v>
+      </c>
     </row>
     <row r="61" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C61" s="10">
         <v>3020</v>
@@ -8341,15 +8787,19 @@
       <c r="AB61" s="10">
         <v>128065</v>
       </c>
-      <c r="AC61" s="10"/>
-      <c r="AD61" s="10"/>
+      <c r="AC61" s="10">
+        <v>318992</v>
+      </c>
+      <c r="AD61" s="10">
+        <v>72908</v>
+      </c>
     </row>
     <row r="62" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C62" s="10">
         <v>255</v>
@@ -8388,7 +8838,7 @@
         <v>2136</v>
       </c>
       <c r="O62" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="P62" s="10">
         <v>9141</v>
@@ -8429,15 +8879,19 @@
       <c r="AB62" s="10">
         <v>15159</v>
       </c>
-      <c r="AC62" s="10"/>
-      <c r="AD62" s="10"/>
+      <c r="AC62" s="10">
+        <v>47133</v>
+      </c>
+      <c r="AD62" s="10">
+        <v>5060</v>
+      </c>
     </row>
     <row r="63" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C63" s="10">
         <v>1611</v>
@@ -8473,10 +8927,10 @@
         <v>176934</v>
       </c>
       <c r="N63" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="O63" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="P63" s="10">
         <v>84516</v>
@@ -8517,15 +8971,19 @@
       <c r="AB63" s="10">
         <v>74958</v>
       </c>
-      <c r="AC63" s="10"/>
-      <c r="AD63" s="10"/>
+      <c r="AC63" s="10">
+        <v>205538</v>
+      </c>
+      <c r="AD63" s="10">
+        <v>26470</v>
+      </c>
     </row>
     <row r="64" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C64" s="10">
         <v>490</v>
@@ -8576,7 +9034,7 @@
         <v>4263</v>
       </c>
       <c r="S64" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="T64" s="10">
         <v>16209</v>
@@ -8605,15 +9063,19 @@
       <c r="AB64" s="10">
         <v>18543</v>
       </c>
-      <c r="AC64" s="10"/>
-      <c r="AD64" s="10"/>
+      <c r="AC64" s="10">
+        <v>63492</v>
+      </c>
+      <c r="AD64" s="10">
+        <v>6916</v>
+      </c>
     </row>
     <row r="65" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A65" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C65" s="10">
         <v>721</v>
@@ -8640,7 +9102,7 @@
         <v>1769</v>
       </c>
       <c r="K65" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="L65" s="10">
         <v>4697</v>
@@ -8661,10 +9123,10 @@
         <v>55460</v>
       </c>
       <c r="R65" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="S65" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="T65" s="10">
         <v>17325</v>
@@ -8693,15 +9155,19 @@
       <c r="AB65" s="10">
         <v>19983</v>
       </c>
-      <c r="AC65" s="10"/>
-      <c r="AD65" s="10"/>
+      <c r="AC65" s="10">
+        <v>60585</v>
+      </c>
+      <c r="AD65" s="10">
+        <v>7842</v>
+      </c>
     </row>
     <row r="66" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A66" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C66" s="10">
         <v>4247</v>
@@ -8740,7 +9206,7 @@
         <v>104726</v>
       </c>
       <c r="O66" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="P66" s="10">
         <v>251729</v>
@@ -8755,7 +9221,7 @@
         <v>9522</v>
       </c>
       <c r="T66" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="U66" s="10">
         <v>665850</v>
@@ -8781,15 +9247,19 @@
       <c r="AB66" s="10">
         <v>369379</v>
       </c>
-      <c r="AC66" s="10"/>
-      <c r="AD66" s="10"/>
+      <c r="AC66" s="10">
+        <v>855865</v>
+      </c>
+      <c r="AD66" s="10">
+        <v>193997</v>
+      </c>
     </row>
     <row r="67" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A67" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C67" s="10">
         <v>152</v>
@@ -8869,15 +9339,19 @@
       <c r="AB67" s="10">
         <v>2611</v>
       </c>
-      <c r="AC67" s="10"/>
-      <c r="AD67" s="10"/>
+      <c r="AC67" s="10">
+        <v>8527</v>
+      </c>
+      <c r="AD67" s="10">
+        <v>1283</v>
+      </c>
     </row>
     <row r="68" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A68" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B68" s="1" t="s">
         <v>78</v>
-      </c>
-      <c r="B68" s="1" t="s">
-        <v>79</v>
       </c>
       <c r="C68" s="10">
         <v>5998</v>
@@ -8916,7 +9390,7 @@
         <v>85273</v>
       </c>
       <c r="O68" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="P68" s="10">
         <v>190968</v>
@@ -8957,15 +9431,19 @@
       <c r="AB68" s="10">
         <v>272594</v>
       </c>
-      <c r="AC68" s="10"/>
-      <c r="AD68" s="10"/>
+      <c r="AC68" s="10">
+        <v>608420</v>
+      </c>
+      <c r="AD68" s="10">
+        <v>150084</v>
+      </c>
     </row>
     <row r="69" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A69" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C69" s="10">
         <v>2054</v>
@@ -8995,13 +9473,13 @@
         <v>1115</v>
       </c>
       <c r="L69" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M69" s="10">
         <v>145687</v>
       </c>
       <c r="N69" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="O69" s="10">
         <v>4929</v>
@@ -9028,7 +9506,7 @@
         <v>48666</v>
       </c>
       <c r="W69" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="X69" s="10">
         <v>92519</v>
@@ -9045,15 +9523,19 @@
       <c r="AB69" s="10">
         <v>98793</v>
       </c>
-      <c r="AC69" s="10"/>
-      <c r="AD69" s="10"/>
+      <c r="AC69" s="10">
+        <v>233888</v>
+      </c>
+      <c r="AD69" s="10">
+        <v>57871</v>
+      </c>
     </row>
     <row r="70" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A70" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C70" s="10">
         <v>3242</v>
@@ -9133,15 +9615,19 @@
       <c r="AB70" s="10">
         <v>99417</v>
       </c>
-      <c r="AC70" s="10"/>
-      <c r="AD70" s="10"/>
+      <c r="AC70" s="10">
+        <v>229257</v>
+      </c>
+      <c r="AD70" s="10">
+        <v>57537</v>
+      </c>
     </row>
     <row r="71" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C71" s="10">
         <v>7502</v>
@@ -9180,7 +9666,7 @@
         <v>45136</v>
       </c>
       <c r="O71" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="P71" s="10">
         <v>118142</v>
@@ -9221,14 +9707,18 @@
       <c r="AB71" s="10">
         <v>147238</v>
       </c>
-      <c r="AC71" s="10"/>
-      <c r="AD71" s="10"/>
-    </row>
-    <row r="72" spans="1:30" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="34" t="s">
-        <v>83</v>
-      </c>
-      <c r="B72" s="34"/>
+      <c r="AC71" s="10">
+        <v>333809</v>
+      </c>
+      <c r="AD71" s="10">
+        <v>81670</v>
+      </c>
+    </row>
+    <row r="72" spans="1:30" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="36" t="s">
+        <v>82</v>
+      </c>
+      <c r="B72" s="36"/>
       <c r="C72" s="11">
         <v>268412</v>
       </c>
@@ -9307,42 +9797,46 @@
       <c r="AB72" s="11">
         <v>2976884</v>
       </c>
-      <c r="AC72" s="11"/>
-      <c r="AD72" s="11"/>
+      <c r="AC72" s="11">
+        <v>6602632</v>
+      </c>
+      <c r="AD72" s="11">
+        <v>1698231</v>
+      </c>
     </row>
     <row r="73" spans="1:30" x14ac:dyDescent="0.3">
       <c r="D73" s="14"/>
       <c r="E73" s="14"/>
     </row>
     <row r="74" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A74" s="21" t="s">
-        <v>93</v>
-      </c>
-      <c r="B74" s="21"/>
+      <c r="A74" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="B74" s="22"/>
       <c r="D74" s="14"/>
     </row>
-    <row r="75" spans="1:30" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="28" t="s">
-        <v>115</v>
-      </c>
-      <c r="B75" s="28"/>
-      <c r="C75" s="28"/>
-      <c r="D75" s="28"/>
-      <c r="E75" s="28"/>
-      <c r="F75" s="28"/>
+    <row r="75" spans="1:30" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A75" s="26" t="s">
+        <v>114</v>
+      </c>
+      <c r="B75" s="26"/>
+      <c r="C75" s="26"/>
+      <c r="D75" s="26"/>
+      <c r="E75" s="26"/>
+      <c r="F75" s="26"/>
       <c r="G75" s="4"/>
       <c r="H75" s="4"/>
       <c r="I75" s="4"/>
       <c r="J75" s="4"/>
       <c r="K75" s="4"/>
     </row>
-    <row r="76" spans="1:30" ht="58.7" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="28"/>
-      <c r="B76" s="28"/>
-      <c r="C76" s="28"/>
-      <c r="D76" s="28"/>
-      <c r="E76" s="28"/>
-      <c r="F76" s="28"/>
+    <row r="76" spans="1:30" ht="58.65" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="26"/>
+      <c r="B76" s="26"/>
+      <c r="C76" s="26"/>
+      <c r="D76" s="26"/>
+      <c r="E76" s="26"/>
+      <c r="F76" s="26"/>
       <c r="G76" s="4"/>
       <c r="H76" s="4"/>
       <c r="I76" s="4"/>
@@ -9350,14 +9844,14 @@
       <c r="K76" s="4"/>
     </row>
     <row r="77" spans="1:30" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="20" t="s">
-        <v>104</v>
-      </c>
-      <c r="B77" s="20"/>
-      <c r="C77" s="20"/>
-      <c r="D77" s="20"/>
-      <c r="E77" s="20"/>
-      <c r="F77" s="20"/>
+      <c r="A77" s="21" t="s">
+        <v>103</v>
+      </c>
+      <c r="B77" s="21"/>
+      <c r="C77" s="21"/>
+      <c r="D77" s="21"/>
+      <c r="E77" s="21"/>
+      <c r="F77" s="21"/>
       <c r="G77" s="4"/>
       <c r="H77" s="4"/>
       <c r="I77" s="4"/>
@@ -9365,19 +9859,19 @@
       <c r="K77" s="4"/>
     </row>
     <row r="78" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A78" s="19" t="s">
-        <v>103</v>
-      </c>
-      <c r="B78" s="20"/>
-      <c r="C78" s="20"/>
-      <c r="D78" s="20"/>
-      <c r="E78" s="20"/>
-      <c r="F78" s="20"/>
-      <c r="G78" s="20"/>
-      <c r="H78" s="20"/>
-      <c r="I78" s="20"/>
-      <c r="J78" s="20"/>
-      <c r="K78" s="20"/>
+      <c r="A78" s="20" t="s">
+        <v>102</v>
+      </c>
+      <c r="B78" s="21"/>
+      <c r="C78" s="21"/>
+      <c r="D78" s="21"/>
+      <c r="E78" s="21"/>
+      <c r="F78" s="21"/>
+      <c r="G78" s="21"/>
+      <c r="H78" s="21"/>
+      <c r="I78" s="21"/>
+      <c r="J78" s="21"/>
+      <c r="K78" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -9397,7 +9891,4 @@
   <pageMargins left="0.26" right="0.19" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="62" fitToHeight="0" orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=customMetadata/metadata.xml><?xml version="1.0" encoding="utf-8" standalone="yes"?><metadata xmlns:m="http://www.titus.com/ns/Greek Statistic Authority" id="13a77cc9-12d1-427b-8d7b-f38fa1de31a1"><m:Classification value="Internal"><alt>Classification=Internal</alt></m:Classification></metadata>
 </file>
</xml_diff>